<commit_message>
two sum completed for GO
</commit_message>
<xml_diff>
--- a/blind-75/go/blind-75-go.xlsx
+++ b/blind-75/go/blind-75-go.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C7F2B0-95C1-404A-A330-3574BC64A64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Tracker" state="visible" r:id="rId4"/>
+    <sheet name="Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="223">
   <si>
     <t>Overall Completion:</t>
   </si>
@@ -677,42 +681,56 @@
   </si>
   <si>
     <t>Graph Valid Tree</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="11"/>
+      <color rgb="FF00B8A3"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FFFFC01E"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF00B8A3"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0563C1"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFC01E"/>
-    </font>
-    <font>
-      <b/>
+      <sz val="11"/>
       <color rgb="FFFF375F"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1092,9 +1110,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G78"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -1105,15 +1123,16 @@
     <col min="7" max="7" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2">
         <f>COUNTIF(F4:F78, "Completed")/75</f>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>1.3333333333333334E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1136,7 +1155,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1153,10 +1172,10 @@
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1176,7 +1195,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1196,7 +1215,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1216,7 +1235,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1236,7 +1255,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1256,7 +1275,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -1276,7 +1295,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1296,7 +1315,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -1316,7 +1335,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1336,7 +1355,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -1356,7 +1375,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -1376,7 +1395,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>49</v>
       </c>
@@ -1396,7 +1415,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -1416,7 +1435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -1436,7 +1455,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>58</v>
       </c>
@@ -1456,7 +1475,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -1476,7 +1495,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -1496,7 +1515,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -1516,7 +1535,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>70</v>
       </c>
@@ -1536,7 +1555,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>73</v>
       </c>
@@ -1556,7 +1575,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -1576,7 +1595,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>78</v>
       </c>
@@ -1596,7 +1615,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>81</v>
       </c>
@@ -1616,7 +1635,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -1636,7 +1655,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>87</v>
       </c>
@@ -1656,7 +1675,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>90</v>
       </c>
@@ -1676,7 +1695,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>93</v>
       </c>
@@ -1696,7 +1715,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>95</v>
       </c>
@@ -1716,7 +1735,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>98</v>
       </c>
@@ -1736,7 +1755,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>101</v>
       </c>
@@ -1756,7 +1775,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>104</v>
       </c>
@@ -1776,7 +1795,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>107</v>
       </c>
@@ -1796,7 +1815,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>110</v>
       </c>
@@ -1816,7 +1835,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>113</v>
       </c>
@@ -1836,7 +1855,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>116</v>
       </c>
@@ -1856,7 +1875,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>119</v>
       </c>
@@ -1876,7 +1895,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>122</v>
       </c>
@@ -1896,7 +1915,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>124</v>
       </c>
@@ -1916,7 +1935,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>126</v>
       </c>
@@ -1936,7 +1955,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>129</v>
       </c>
@@ -1956,7 +1975,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>131</v>
       </c>
@@ -1976,7 +1995,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>133</v>
       </c>
@@ -1996,7 +2015,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>136</v>
       </c>
@@ -2016,7 +2035,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>138</v>
       </c>
@@ -2036,7 +2055,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>141</v>
       </c>
@@ -2056,7 +2075,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>144</v>
       </c>
@@ -2076,7 +2095,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>147</v>
       </c>
@@ -2096,7 +2115,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>150</v>
       </c>
@@ -2116,7 +2135,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>152</v>
       </c>
@@ -2136,7 +2155,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>155</v>
       </c>
@@ -2156,7 +2175,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>157</v>
       </c>
@@ -2176,7 +2195,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>159</v>
       </c>
@@ -2196,7 +2215,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>161</v>
       </c>
@@ -2216,7 +2235,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>164</v>
       </c>
@@ -2236,7 +2255,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>167</v>
       </c>
@@ -2256,7 +2275,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>170</v>
       </c>
@@ -2276,7 +2295,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>173</v>
       </c>
@@ -2296,7 +2315,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>176</v>
       </c>
@@ -2316,7 +2335,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>179</v>
       </c>
@@ -2336,7 +2355,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>182</v>
       </c>
@@ -2356,7 +2375,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>185</v>
       </c>
@@ -2376,7 +2395,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>188</v>
       </c>
@@ -2396,7 +2415,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>191</v>
       </c>
@@ -2416,7 +2435,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>194</v>
       </c>
@@ -2436,7 +2455,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>197</v>
       </c>
@@ -2456,7 +2475,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>200</v>
       </c>
@@ -2476,7 +2495,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>202</v>
       </c>
@@ -2496,7 +2515,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>205</v>
       </c>
@@ -2516,7 +2535,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>208</v>
       </c>
@@ -2536,7 +2555,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>211</v>
       </c>
@@ -2556,7 +2575,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>213</v>
       </c>
@@ -2576,7 +2595,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>215</v>
       </c>
@@ -2596,7 +2615,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>217</v>
       </c>
@@ -2616,7 +2635,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>220</v>
       </c>
@@ -2637,92 +2656,89 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F10:F78">
-      <formula1>"Not Started,In progress,Completed,Needs Review"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F4:F78">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F4:F78" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In progress,Completed,Needs Review"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E4" r:id="rId1" tooltip="https://leetcode.com/problems/two-sum"/>
-    <hyperlink ref="E5" r:id="rId2" tooltip="https://leetcode.com/problems/longest-substring-without-repeating-characters"/>
-    <hyperlink ref="E6" r:id="rId3" tooltip="https://leetcode.com/problems/longest-palindromic-substring"/>
-    <hyperlink ref="E7" r:id="rId4" tooltip="https://leetcode.com/problems/container-with-most-water"/>
-    <hyperlink ref="E8" r:id="rId5" tooltip="https://leetcode.com/problems/3sum"/>
-    <hyperlink ref="E9" r:id="rId6" tooltip="https://leetcode.com/problems/remove-nth-node-from-end-of-list"/>
-    <hyperlink ref="E10" r:id="rId7" tooltip="https://leetcode.com/problems/valid-parentheses"/>
-    <hyperlink ref="E11" r:id="rId8" tooltip="https://leetcode.com/problems/merge-two-sorted-lists"/>
-    <hyperlink ref="E12" r:id="rId9" tooltip="https://leetcode.com/problems/merge-k-sorted-lists"/>
-    <hyperlink ref="E13" r:id="rId10" tooltip="https://leetcode.com/problems/search-in-rotated-sorted-array"/>
-    <hyperlink ref="E14" r:id="rId11" tooltip="https://leetcode.com/problems/combination-sum"/>
-    <hyperlink ref="E15" r:id="rId12" tooltip="https://leetcode.com/problems/rotate-image"/>
-    <hyperlink ref="E16" r:id="rId13" tooltip="https://leetcode.com/problems/group-anagrams"/>
-    <hyperlink ref="E17" r:id="rId14" tooltip="https://leetcode.com/problems/maximum-subarray"/>
-    <hyperlink ref="E18" r:id="rId15" tooltip="https://leetcode.com/problems/spiral-matrix"/>
-    <hyperlink ref="E19" r:id="rId16" tooltip="https://leetcode.com/problems/jump-game"/>
-    <hyperlink ref="E20" r:id="rId17" tooltip="https://leetcode.com/problems/merge-intervals"/>
-    <hyperlink ref="E21" r:id="rId18" tooltip="https://leetcode.com/problems/insert-interval"/>
-    <hyperlink ref="E22" r:id="rId19" tooltip="https://leetcode.com/problems/unique-paths"/>
-    <hyperlink ref="E23" r:id="rId20" tooltip="https://leetcode.com/problems/climbing-stairs"/>
-    <hyperlink ref="E24" r:id="rId21" tooltip="https://leetcode.com/problems/set-matrix-zeroes"/>
-    <hyperlink ref="E25" r:id="rId22" tooltip="https://leetcode.com/problems/minimum-window-substring"/>
-    <hyperlink ref="E26" r:id="rId23" tooltip="https://leetcode.com/problems/word-search"/>
-    <hyperlink ref="E27" r:id="rId24" tooltip="https://leetcode.com/problems/decode-ways"/>
-    <hyperlink ref="E28" r:id="rId25" tooltip="https://leetcode.com/problems/validate-binary-search-tree"/>
-    <hyperlink ref="E29" r:id="rId26" tooltip="https://leetcode.com/problems/same-tree"/>
-    <hyperlink ref="E30" r:id="rId27" tooltip="https://leetcode.com/problems/binary-tree-level-order-traversal"/>
-    <hyperlink ref="E31" r:id="rId28" tooltip="https://leetcode.com/problems/maximum-depth-of-binary-tree"/>
-    <hyperlink ref="E32" r:id="rId29" tooltip="https://leetcode.com/problems/construct-binary-tree-from-preorder-and-inorder-traversal"/>
-    <hyperlink ref="E33" r:id="rId30" tooltip="https://leetcode.com/problems/best-time-to-buy-and-sell-stock"/>
-    <hyperlink ref="E34" r:id="rId31" tooltip="https://leetcode.com/problems/binary-tree-maximum-path-sum"/>
-    <hyperlink ref="E35" r:id="rId32" tooltip="https://leetcode.com/problems/valid-palindrome"/>
-    <hyperlink ref="E36" r:id="rId33" tooltip="https://leetcode.com/problems/longest-consecutive-sequence"/>
-    <hyperlink ref="E37" r:id="rId34" tooltip="https://leetcode.com/problems/clone-graph"/>
-    <hyperlink ref="E38" r:id="rId35" tooltip="https://leetcode.com/problems/word-break"/>
-    <hyperlink ref="E39" r:id="rId36" tooltip="https://leetcode.com/problems/linked-list-cycle"/>
-    <hyperlink ref="E40" r:id="rId37" tooltip="https://leetcode.com/problems/reorder-list"/>
-    <hyperlink ref="E41" r:id="rId38" tooltip="https://leetcode.com/problems/maximum-product-subarray"/>
-    <hyperlink ref="E42" r:id="rId39" tooltip="https://leetcode.com/problems/find-minimum-in-rotated-sorted-array"/>
-    <hyperlink ref="E43" r:id="rId40" tooltip="https://leetcode.com/problems/reverse-bits"/>
-    <hyperlink ref="E44" r:id="rId41" tooltip="https://leetcode.com/problems/number-of-1-bits"/>
-    <hyperlink ref="E45" r:id="rId42" tooltip="https://leetcode.com/problems/house-robber"/>
-    <hyperlink ref="E46" r:id="rId43" tooltip="https://leetcode.com/problems/number-of-islands"/>
-    <hyperlink ref="E47" r:id="rId44" tooltip="https://leetcode.com/problems/reverse-linked-list"/>
-    <hyperlink ref="E48" r:id="rId45" tooltip="https://leetcode.com/problems/course-schedule"/>
-    <hyperlink ref="E49" r:id="rId46" tooltip="https://leetcode.com/problems/implement-trie-prefix-tree"/>
-    <hyperlink ref="E50" r:id="rId47" tooltip="https://leetcode.com/problems/design-add-and-search-words-data-structure"/>
-    <hyperlink ref="E51" r:id="rId48" tooltip="https://leetcode.com/problems/word-search-ii"/>
-    <hyperlink ref="E52" r:id="rId49" tooltip="https://leetcode.com/problems/house-robber-ii"/>
-    <hyperlink ref="E53" r:id="rId50" tooltip="https://leetcode.com/problems/contains-duplicate"/>
-    <hyperlink ref="E54" r:id="rId51" tooltip="https://leetcode.com/problems/invert-binary-tree"/>
-    <hyperlink ref="E55" r:id="rId52" tooltip="https://leetcode.com/problems/kth-smallest-element-in-a-bst"/>
-    <hyperlink ref="E56" r:id="rId53" tooltip="https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree"/>
-    <hyperlink ref="E57" r:id="rId54" tooltip="https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-tree"/>
-    <hyperlink ref="E58" r:id="rId55" tooltip="https://leetcode.com/problems/product-of-array-except-self"/>
-    <hyperlink ref="E59" r:id="rId56" tooltip="https://leetcode.com/problems/missing-number"/>
-    <hyperlink ref="E60" r:id="rId57" tooltip="https://leetcode.com/problems/alien-dictionary"/>
-    <hyperlink ref="E61" r:id="rId58" tooltip="https://leetcode.com/problems/encode-and-decode-strings"/>
-    <hyperlink ref="E62" r:id="rId59" tooltip="https://leetcode.com/problems/find-median-from-data-stream"/>
-    <hyperlink ref="E63" r:id="rId60" tooltip="https://leetcode.com/problems/longest-increasing-subsequence"/>
-    <hyperlink ref="E64" r:id="rId61" tooltip="https://leetcode.com/problems/coin-change"/>
-    <hyperlink ref="E65" r:id="rId62" tooltip="https://leetcode.com/problems/number-of-connected-components-in-an-undirected-graph"/>
-    <hyperlink ref="E66" r:id="rId63" tooltip="https://leetcode.com/problems/counting-bits"/>
-    <hyperlink ref="E67" r:id="rId64" tooltip="https://leetcode.com/problems/top-k-frequent-elements"/>
-    <hyperlink ref="E68" r:id="rId65" tooltip="https://leetcode.com/problems/sum-of-two-integers"/>
-    <hyperlink ref="E69" r:id="rId66" tooltip="https://leetcode.com/problems/pacific-atlantic-water-flow"/>
-    <hyperlink ref="E70" r:id="rId67" tooltip="https://leetcode.com/problems/longest-repeating-character-replacement"/>
-    <hyperlink ref="E71" r:id="rId68" tooltip="https://leetcode.com/problems/non-overlapping-intervals"/>
-    <hyperlink ref="E72" r:id="rId69" tooltip="https://leetcode.com/problems/serialize-and-deserialize-bst"/>
-    <hyperlink ref="E73" r:id="rId70" tooltip="https://leetcode.com/problems/subtree-of-another-tree"/>
-    <hyperlink ref="E74" r:id="rId71" tooltip="https://leetcode.com/problems/palindromic-substrings"/>
-    <hyperlink ref="E75" r:id="rId72" tooltip="https://leetcode.com/problems/longest-common-subsequence"/>
-    <hyperlink ref="E76" r:id="rId73" tooltip="https://leetcode.com/problems/meeting-rooms"/>
-    <hyperlink ref="E77" r:id="rId74" tooltip="https://leetcode.com/problems/meeting-rooms-ii"/>
-    <hyperlink ref="E78" r:id="rId75" tooltip="https://leetcode.com/problems/graph-valid-tree"/>
+    <hyperlink ref="E4" r:id="rId1" tooltip="https://leetcode.com/problems/two-sum" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="E5" r:id="rId2" tooltip="https://leetcode.com/problems/longest-substring-without-repeating-characters" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E6" r:id="rId3" tooltip="https://leetcode.com/problems/longest-palindromic-substring" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E7" r:id="rId4" tooltip="https://leetcode.com/problems/container-with-most-water" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E8" r:id="rId5" tooltip="https://leetcode.com/problems/3sum" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E9" r:id="rId6" tooltip="https://leetcode.com/problems/remove-nth-node-from-end-of-list" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E10" r:id="rId7" tooltip="https://leetcode.com/problems/valid-parentheses" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="E11" r:id="rId8" tooltip="https://leetcode.com/problems/merge-two-sorted-lists" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E12" r:id="rId9" tooltip="https://leetcode.com/problems/merge-k-sorted-lists" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="E13" r:id="rId10" tooltip="https://leetcode.com/problems/search-in-rotated-sorted-array" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E14" r:id="rId11" tooltip="https://leetcode.com/problems/combination-sum" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E15" r:id="rId12" tooltip="https://leetcode.com/problems/rotate-image" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E16" r:id="rId13" tooltip="https://leetcode.com/problems/group-anagrams" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E17" r:id="rId14" tooltip="https://leetcode.com/problems/maximum-subarray" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E18" r:id="rId15" tooltip="https://leetcode.com/problems/spiral-matrix" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E19" r:id="rId16" tooltip="https://leetcode.com/problems/jump-game" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E20" r:id="rId17" tooltip="https://leetcode.com/problems/merge-intervals" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E21" r:id="rId18" tooltip="https://leetcode.com/problems/insert-interval" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E22" r:id="rId19" tooltip="https://leetcode.com/problems/unique-paths" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E23" r:id="rId20" tooltip="https://leetcode.com/problems/climbing-stairs" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E24" r:id="rId21" tooltip="https://leetcode.com/problems/set-matrix-zeroes" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E25" r:id="rId22" tooltip="https://leetcode.com/problems/minimum-window-substring" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="E26" r:id="rId23" tooltip="https://leetcode.com/problems/word-search" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="E27" r:id="rId24" tooltip="https://leetcode.com/problems/decode-ways" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="E28" r:id="rId25" tooltip="https://leetcode.com/problems/validate-binary-search-tree" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E29" r:id="rId26" tooltip="https://leetcode.com/problems/same-tree" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E30" r:id="rId27" tooltip="https://leetcode.com/problems/binary-tree-level-order-traversal" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E31" r:id="rId28" tooltip="https://leetcode.com/problems/maximum-depth-of-binary-tree" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E32" r:id="rId29" tooltip="https://leetcode.com/problems/construct-binary-tree-from-preorder-and-inorder-traversal" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="E33" r:id="rId30" tooltip="https://leetcode.com/problems/best-time-to-buy-and-sell-stock" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="E34" r:id="rId31" tooltip="https://leetcode.com/problems/binary-tree-maximum-path-sum" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="E35" r:id="rId32" tooltip="https://leetcode.com/problems/valid-palindrome" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="E36" r:id="rId33" tooltip="https://leetcode.com/problems/longest-consecutive-sequence" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="E37" r:id="rId34" tooltip="https://leetcode.com/problems/clone-graph" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="E38" r:id="rId35" tooltip="https://leetcode.com/problems/word-break" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="E39" r:id="rId36" tooltip="https://leetcode.com/problems/linked-list-cycle" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="E40" r:id="rId37" tooltip="https://leetcode.com/problems/reorder-list" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="E41" r:id="rId38" tooltip="https://leetcode.com/problems/maximum-product-subarray" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="E42" r:id="rId39" tooltip="https://leetcode.com/problems/find-minimum-in-rotated-sorted-array" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="E43" r:id="rId40" tooltip="https://leetcode.com/problems/reverse-bits" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="E44" r:id="rId41" tooltip="https://leetcode.com/problems/number-of-1-bits" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="E45" r:id="rId42" tooltip="https://leetcode.com/problems/house-robber" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="E46" r:id="rId43" tooltip="https://leetcode.com/problems/number-of-islands" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="E47" r:id="rId44" tooltip="https://leetcode.com/problems/reverse-linked-list" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="E48" r:id="rId45" tooltip="https://leetcode.com/problems/course-schedule" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="E49" r:id="rId46" tooltip="https://leetcode.com/problems/implement-trie-prefix-tree" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="E50" r:id="rId47" tooltip="https://leetcode.com/problems/design-add-and-search-words-data-structure" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="E51" r:id="rId48" tooltip="https://leetcode.com/problems/word-search-ii" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="E52" r:id="rId49" tooltip="https://leetcode.com/problems/house-robber-ii" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="E53" r:id="rId50" tooltip="https://leetcode.com/problems/contains-duplicate" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="E54" r:id="rId51" tooltip="https://leetcode.com/problems/invert-binary-tree" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="E55" r:id="rId52" tooltip="https://leetcode.com/problems/kth-smallest-element-in-a-bst" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="E56" r:id="rId53" tooltip="https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="E57" r:id="rId54" tooltip="https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-tree" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="E58" r:id="rId55" tooltip="https://leetcode.com/problems/product-of-array-except-self" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="E59" r:id="rId56" tooltip="https://leetcode.com/problems/missing-number" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="E60" r:id="rId57" tooltip="https://leetcode.com/problems/alien-dictionary" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="E61" r:id="rId58" tooltip="https://leetcode.com/problems/encode-and-decode-strings" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="E62" r:id="rId59" tooltip="https://leetcode.com/problems/find-median-from-data-stream" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="E63" r:id="rId60" tooltip="https://leetcode.com/problems/longest-increasing-subsequence" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="E64" r:id="rId61" tooltip="https://leetcode.com/problems/coin-change" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="E65" r:id="rId62" tooltip="https://leetcode.com/problems/number-of-connected-components-in-an-undirected-graph" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="E66" r:id="rId63" tooltip="https://leetcode.com/problems/counting-bits" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="E67" r:id="rId64" tooltip="https://leetcode.com/problems/top-k-frequent-elements" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="E68" r:id="rId65" tooltip="https://leetcode.com/problems/sum-of-two-integers" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="E69" r:id="rId66" tooltip="https://leetcode.com/problems/pacific-atlantic-water-flow" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="E70" r:id="rId67" tooltip="https://leetcode.com/problems/longest-repeating-character-replacement" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="E71" r:id="rId68" tooltip="https://leetcode.com/problems/non-overlapping-intervals" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="E72" r:id="rId69" tooltip="https://leetcode.com/problems/serialize-and-deserialize-bst" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="E73" r:id="rId70" tooltip="https://leetcode.com/problems/subtree-of-another-tree" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="E74" r:id="rId71" tooltip="https://leetcode.com/problems/palindromic-substrings" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="E75" r:id="rId72" tooltip="https://leetcode.com/problems/longest-common-subsequence" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="E76" r:id="rId73" tooltip="https://leetcode.com/problems/meeting-rooms" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="E77" r:id="rId74" tooltip="https://leetcode.com/problems/meeting-rooms-ii" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="E78" r:id="rId75" tooltip="https://leetcode.com/problems/graph-valid-tree" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
valid parenthesis completed for GO
</commit_message>
<xml_diff>
--- a/blind-75/go/blind-75-go.xlsx
+++ b/blind-75/go/blind-75-go.xlsx
@@ -3,13 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C7F2B0-95C1-404A-A330-3574BC64A64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67BE9898-6C7F-4F0C-AED4-0000857494AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tracker!$A$3:$G$78</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
@@ -1111,6 +1114,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G78"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1129,7 +1133,7 @@
       </c>
       <c r="B1" s="2">
         <f>COUNTIF(F4:F78, "Completed")/75</f>
-        <v>1.3333333333333334E-2</v>
+        <v>2.6666666666666668E-2</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
@@ -1175,7 +1179,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1195,7 +1199,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1215,7 +1219,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1235,7 +1239,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1255,7 +1259,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1292,7 +1296,7 @@
         <v>12</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -1315,7 +1319,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -1335,7 +1339,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -1355,7 +1359,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -1375,7 +1379,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -1395,7 +1399,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>49</v>
       </c>
@@ -1415,7 +1419,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -1435,7 +1439,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>55</v>
       </c>
@@ -1455,7 +1459,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>58</v>
       </c>
@@ -1475,7 +1479,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -1495,7 +1499,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -1515,7 +1519,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -1555,7 +1559,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>73</v>
       </c>
@@ -1575,7 +1579,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -1595,7 +1599,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>78</v>
       </c>
@@ -1615,7 +1619,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>81</v>
       </c>
@@ -1635,7 +1639,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>84</v>
       </c>
@@ -1675,7 +1679,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>90</v>
       </c>
@@ -1715,7 +1719,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>95</v>
       </c>
@@ -1755,7 +1759,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>101</v>
       </c>
@@ -1795,7 +1799,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>107</v>
       </c>
@@ -1815,7 +1819,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>110</v>
       </c>
@@ -1835,7 +1839,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>113</v>
       </c>
@@ -1875,7 +1879,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>119</v>
       </c>
@@ -1895,7 +1899,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>122</v>
       </c>
@@ -1915,7 +1919,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>124</v>
       </c>
@@ -1975,7 +1979,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>131</v>
       </c>
@@ -1995,7 +1999,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>133</v>
       </c>
@@ -2035,7 +2039,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>138</v>
       </c>
@@ -2055,7 +2059,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>141</v>
       </c>
@@ -2075,7 +2079,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>144</v>
       </c>
@@ -2095,7 +2099,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>147</v>
       </c>
@@ -2115,7 +2119,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>150</v>
       </c>
@@ -2175,7 +2179,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>157</v>
       </c>
@@ -2195,7 +2199,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>159</v>
       </c>
@@ -2215,7 +2219,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>161</v>
       </c>
@@ -2235,7 +2239,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>164</v>
       </c>
@@ -2275,7 +2279,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>170</v>
       </c>
@@ -2295,7 +2299,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>173</v>
       </c>
@@ -2315,7 +2319,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>176</v>
       </c>
@@ -2335,7 +2339,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>179</v>
       </c>
@@ -2355,7 +2359,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>182</v>
       </c>
@@ -2375,7 +2379,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>185</v>
       </c>
@@ -2415,7 +2419,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>191</v>
       </c>
@@ -2435,7 +2439,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>194</v>
       </c>
@@ -2455,7 +2459,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>197</v>
       </c>
@@ -2475,7 +2479,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>200</v>
       </c>
@@ -2495,7 +2499,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>202</v>
       </c>
@@ -2515,7 +2519,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>205</v>
       </c>
@@ -2555,7 +2559,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>211</v>
       </c>
@@ -2575,7 +2579,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>213</v>
       </c>
@@ -2615,7 +2619,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>217</v>
       </c>
@@ -2635,7 +2639,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>220</v>
       </c>
@@ -2656,6 +2660,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:G78" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="Easy"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F4:F78" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In progress,Completed,Needs Review"</formula1>

</xml_diff>

<commit_message>
Added solution for merge two lists
</commit_message>
<xml_diff>
--- a/blind-75/go/blind-75-go.xlsx
+++ b/blind-75/go/blind-75-go.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67BE9898-6C7F-4F0C-AED4-0000857494AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70579828-A4A7-41FD-97D9-C7FF94CCAD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="B1" s="2">
         <f>COUNTIF(F4:F78, "Completed")/75</f>
-        <v>2.6666666666666668E-2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
@@ -1316,7 +1316,7 @@
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added solution for climbing stairs
</commit_message>
<xml_diff>
--- a/blind-75/go/blind-75-go.xlsx
+++ b/blind-75/go/blind-75-go.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70579828-A4A7-41FD-97D9-C7FF94CCAD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6097659B-951D-4295-8D94-2E83C2B91D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="B1" s="2">
         <f>COUNTIF(F4:F78, "Completed")/75</f>
-        <v>0.04</v>
+        <v>5.3333333333333337E-2</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
@@ -1556,7 +1556,7 @@
         <v>12</v>
       </c>
       <c r="F23" t="s">
-        <v>13</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.35">

</xml_diff>